<commit_message>
Pipeline: scrape legacy + contrôle croisé (6Z)
</commit_message>
<xml_diff>
--- a/legacy/Forecast-03072026-6Z.xlsx
+++ b/legacy/Forecast-03072026-6Z.xlsx
@@ -647,7 +647,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 03/07/2026 16:45</t>
+          <t>Généré le : 04/07/2026 08:41</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 03/07/2026 16:45</t>
+          <t>Généré le : 04/07/2026 08:41</t>
         </is>
       </c>
     </row>

</xml_diff>